<commit_message>
NOTIFICATION BAR SLOT OPTION
</commit_message>
<xml_diff>
--- a/backend/Valid_Timetable_Template.xlsx
+++ b/backend/Valid_Timetable_Template.xlsx
@@ -556,8 +556,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>1</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -581,8 +583,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>3</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -606,8 +610,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>5</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -631,8 +637,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>7</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -656,8 +664,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>1</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -681,8 +691,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>3</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -706,8 +718,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>5</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -731,8 +745,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>7</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -756,8 +772,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>1</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -781,8 +799,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>3</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -806,8 +826,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>5</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -831,8 +853,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>7</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -856,8 +880,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>1</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -881,8 +907,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>3</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -906,8 +934,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>5</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -931,8 +961,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>7</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -956,8 +988,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>1</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -981,8 +1015,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>3</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1006,8 +1042,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>5</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1031,8 +1069,10 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>7</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1675,12 +1715,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CSE101_LAB</t>
+          <t>CSE101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Computer Programming Lab</t>
+          <t>CSE Subject 101</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1688,16 +1728,18 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>Theory</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -1719,8 +1761,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1750,8 +1794,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>1</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1781,8 +1827,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1812,8 +1860,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>3</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1843,8 +1893,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>3</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1874,8 +1926,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>3</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1905,8 +1959,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>3</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1936,8 +1992,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>5</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1967,8 +2025,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>5</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1998,8 +2058,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>5</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2029,8 +2091,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>5</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2060,8 +2124,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>7</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2091,8 +2157,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>7</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2122,8 +2190,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>7</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2153,8 +2223,10 @@
           <t>CSE</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>7</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2184,8 +2256,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>1</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2215,8 +2289,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>1</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2246,8 +2322,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>1</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2277,8 +2355,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>1</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2308,8 +2388,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>3</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2339,8 +2421,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>3</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2370,8 +2454,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>3</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2401,8 +2487,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>3</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -2432,8 +2520,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>5</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -2463,8 +2553,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>5</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -2494,8 +2586,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>5</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -2525,8 +2619,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>5</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -2556,8 +2652,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>7</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2587,8 +2685,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D31" t="n">
-        <v>7</v>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2618,8 +2718,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>7</v>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2649,8 +2751,10 @@
           <t>ECE</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>7</v>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2680,8 +2784,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>1</v>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2711,8 +2817,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D35" t="n">
-        <v>1</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2742,8 +2850,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>1</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -2773,8 +2883,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>1</v>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -2804,8 +2916,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>3</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2835,8 +2949,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D39" t="n">
-        <v>3</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -2866,8 +2982,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D40" t="n">
-        <v>3</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -2897,8 +3015,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>3</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -2928,8 +3048,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D42" t="n">
-        <v>5</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -2959,8 +3081,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>5</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2990,8 +3114,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D44" t="n">
-        <v>5</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -3021,8 +3147,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>5</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -3052,8 +3180,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>7</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3083,8 +3213,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D47" t="n">
-        <v>7</v>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -3114,8 +3246,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>7</v>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -3145,8 +3279,10 @@
           <t>EEE</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>7</v>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -3176,8 +3312,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>1</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -3207,8 +3345,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D51" t="n">
-        <v>1</v>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -3238,8 +3378,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D52" t="n">
-        <v>1</v>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -3269,8 +3411,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>1</v>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -3300,8 +3444,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D54" t="n">
-        <v>3</v>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -3331,8 +3477,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D55" t="n">
-        <v>3</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -3362,8 +3510,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D56" t="n">
-        <v>3</v>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -3393,8 +3543,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>3</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -3424,8 +3576,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>5</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -3455,8 +3609,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>5</v>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -3486,8 +3642,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D60" t="n">
-        <v>5</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -3517,8 +3675,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>5</v>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -3548,8 +3708,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>7</v>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -3579,8 +3741,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D63" t="n">
-        <v>7</v>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -3610,8 +3774,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D64" t="n">
-        <v>7</v>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -3641,8 +3807,10 @@
           <t>MECH</t>
         </is>
       </c>
-      <c r="D65" t="n">
-        <v>7</v>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -3672,8 +3840,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D66" t="n">
-        <v>1</v>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -3703,8 +3873,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D67" t="n">
-        <v>1</v>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3734,8 +3906,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D68" t="n">
-        <v>1</v>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -3765,8 +3939,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D69" t="n">
-        <v>1</v>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -3796,8 +3972,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D70" t="n">
-        <v>3</v>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -3827,8 +4005,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D71" t="n">
-        <v>3</v>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3858,8 +4038,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D72" t="n">
-        <v>3</v>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -3889,8 +4071,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D73" t="n">
-        <v>3</v>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -3920,8 +4104,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D74" t="n">
-        <v>5</v>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3951,8 +4137,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D75" t="n">
-        <v>5</v>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3982,8 +4170,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D76" t="n">
-        <v>5</v>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -4013,8 +4203,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D77" t="n">
-        <v>5</v>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -4044,8 +4236,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D78" t="n">
-        <v>7</v>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -4075,8 +4269,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D79" t="n">
-        <v>7</v>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -4106,8 +4302,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D80" t="n">
-        <v>7</v>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -4137,8 +4335,10 @@
           <t>CIVIL</t>
         </is>
       </c>
-      <c r="D81" t="n">
-        <v>7</v>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -4196,7 +4396,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CSE101_LAB</t>
+          <t>CSE101</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4205,7 +4405,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">

</xml_diff>